<commit_message>
Filled out A01_pixell_test_plan_client, and wrote unittest's testing and ensuring all functions of Client class are functioning as intended, also modified spelling and small parts of client.py.
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_client.xlsx
+++ b/tests/A01_pixell_test_plan_client.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dkwarkentin\Documents\Course Folders\2-Intermediate Software Development\Code\Assignments 2024 Spring\Assignment 1\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment_01/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECD6C5C-0BF7-4659-811B-1D416A6C1BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{5ECD6C5C-0BF7-4659-811B-1D416A6C1BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D24A0B50-E7AA-48E0-A4DB-DD89C6733701}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19390" windowHeight="15370" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="53">
   <si>
     <t>Software Development Team - Unit Test Plan</t>
   </si>
@@ -264,13 +264,98 @@
   </si>
   <si>
     <t>Add more rows as necessary</t>
+  </si>
+  <si>
+    <t>Trevor Donald</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>ValueError (""Client Number must be of a numeric type.")</t>
+  </si>
+  <si>
+    <t>ValueError ("Last Name must not be blank.")</t>
+  </si>
+  <si>
+    <t>ValueError ("First Name must not be blank.")</t>
+  </si>
+  <si>
+    <t>EmailNotValidError ("Email Address not valid")</t>
+  </si>
+  <si>
+    <t>self.assertEqual( {input},client._Client _client_number / client.Client_first_name / client._Client_last_name / client._client _email_adress)</t>
+  </si>
+  <si>
+    <t>Initializing the class by calling the class with valid inputs example:      Client(123,"Trevor","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t>Initializing the class by calling the class with invalid inputs example:      Client("123","Trevor","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t>Initializing the class by calling the class with invalid inputs example:      Client(123,"","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t>Initializing the class by calling the class with invalid inputs example:      Client(123,"Trevor","","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t>Initializing the class by calling the class with invalid inputs example:      Client(123,"Trevor","Donald","invalid")</t>
+  </si>
+  <si>
+    <t>After initializing the class calliing the accessor client.client_number</t>
+  </si>
+  <si>
+    <t>After initializing the class calliing the accessor client.first_name</t>
+  </si>
+  <si>
+    <t>After initializing the class calliing the accessor client.last_name</t>
+  </si>
+  <si>
+    <t>After initializing the class calliing the accessor client.email_address</t>
+  </si>
+  <si>
+    <t>After initializing the class calliing the __str__ print(client)</t>
+  </si>
+  <si>
+    <t>self.assertEqual( {input}, self.client.email_adress)</t>
+  </si>
+  <si>
+    <t>self.assertEqual( {input}, self.client.last_name)</t>
+  </si>
+  <si>
+    <t>self.assertEqual( {input}, self.client.first_name)</t>
+  </si>
+  <si>
+    <t>self.assertEqual( {input}, self.client.client_number)</t>
+  </si>
+  <si>
+    <t>self.assertEqual( {input}, str(self.client)</t>
+  </si>
+  <si>
+    <t>with self.assertRaises(ValueError) as context:Client("123", "Trevor", "Donald", "Tdonald35@academic.rrc.ca")
+self.assertEqual(expected, str(context.exception))</t>
+  </si>
+  <si>
+    <t>with self.assertRaises(ValueError) as context:
+            Client(123, "", "Donald", "Tdonald35@academic.rrc.ca")
+        self.assertEqual(expected, str(context.exception))</t>
+  </si>
+  <si>
+    <t>ith self.assertRaises(ValueError) as context:
+            Client(123, "Trevor", "", "Tdonald35@academic.rrc.ca")
+        self.assertEqual(expected, str(context.exception))</t>
+  </si>
+  <si>
+    <t>with self.assertRaises(ValueError) as context:
+            Client(123, "Trevor", "", "Tdonald35@academic.rrc.ca")
+        self.assertEqual(expected, str(context.exception))</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1086,18 +1171,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEBCC4-BB44-48CD-B9AB-1E2FD3EE0EEB}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="29.140625" customWidth="1"/>
-    <col min="6" max="6" width="35.42578125" customWidth="1"/>
-    <col min="7" max="7" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="22.26953125" customWidth="1"/>
+    <col min="4" max="4" width="32.7265625" customWidth="1"/>
+    <col min="5" max="5" width="29.1796875" customWidth="1"/>
+    <col min="6" max="6" width="35.453125" customWidth="1"/>
+    <col min="7" max="7" width="26.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1"/>
-    <row r="2" spans="1:7" ht="73.150000000000006" customHeight="1" thickBot="1">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="1:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="2.15">
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -1109,14 +1194,16 @@
       <c r="F2" s="13"/>
       <c r="G2" s="14"/>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15"/>
+      <c r="C3" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="D3" s="16"/>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
@@ -1125,10 +1212,10 @@
       </c>
       <c r="D4" s="18"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B6" s="10" t="s">
         <v>4</v>
       </c>
@@ -1148,7 +1235,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="66" customHeight="1">
+    <row r="7" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4"/>
       <c r="B7" s="9">
         <v>1</v>
@@ -1159,11 +1246,17 @@
       <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" ht="66" customHeight="1">
+      <c r="E7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4"/>
       <c r="B8" s="11">
         <v>2</v>
@@ -1174,11 +1267,17 @@
       <c r="D8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-    </row>
-    <row r="9" spans="1:7" ht="66" customHeight="1">
+      <c r="E8" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
       <c r="B9" s="11">
         <v>3</v>
@@ -1189,11 +1288,17 @@
       <c r="D9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" spans="1:7" ht="66" customHeight="1">
+      <c r="E9" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="9">
         <v>4</v>
@@ -1204,11 +1309,17 @@
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-    </row>
-    <row r="11" spans="1:7" ht="66" customHeight="1">
+      <c r="E10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="11">
         <v>5</v>
@@ -1219,11 +1330,17 @@
       <c r="D11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>6</v>
       </c>
@@ -1233,11 +1350,17 @@
       <c r="D12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="9">
         <v>7</v>
       </c>
@@ -1247,11 +1370,17 @@
       <c r="D13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-    </row>
-    <row r="14" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="11">
         <v>8</v>
       </c>
@@ -1261,11 +1390,17 @@
       <c r="D14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-    </row>
-    <row r="15" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E14" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="11">
         <v>9</v>
       </c>
@@ -1275,11 +1410,17 @@
       <c r="D15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-    </row>
-    <row r="16" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E15" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="9">
         <v>10</v>
       </c>
@@ -1289,11 +1430,17 @@
       <c r="D16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-    </row>
-    <row r="17" spans="2:7" ht="31.15" customHeight="1">
+      <c r="E16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="11">
         <v>11</v>
       </c>
@@ -1303,7 +1450,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
     </row>
-    <row r="18" spans="2:7" ht="31.15" customHeight="1">
+    <row r="18" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>12</v>
       </c>
@@ -1313,7 +1460,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
     </row>
-    <row r="19" spans="2:7" ht="31.15" customHeight="1">
+    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="9">
         <v>13</v>
       </c>
@@ -1323,7 +1470,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="2:7" ht="31.15" customHeight="1">
+    <row r="20" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="11">
         <v>14</v>
       </c>
@@ -1333,7 +1480,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
     </row>
-    <row r="21" spans="2:7" ht="31.15" customHeight="1">
+    <row r="21" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="11">
         <v>15</v>
       </c>
@@ -1343,7 +1490,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
     </row>
-    <row r="22" spans="2:7" ht="31.15" customHeight="1">
+    <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="9">
         <v>16</v>
       </c>
@@ -1353,7 +1500,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
     </row>
-    <row r="23" spans="2:7" ht="31.15" customHeight="1">
+    <row r="23" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="11">
         <v>17</v>
       </c>
@@ -1363,7 +1510,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="2:7" ht="31.15" customHeight="1">
+    <row r="24" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="11">
         <v>18</v>
       </c>
@@ -1373,7 +1520,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="2:7" ht="31.15" customHeight="1">
+    <row r="25" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="9">
         <v>19</v>
       </c>
@@ -1383,7 +1530,7 @@
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="2:7" ht="31.15" customHeight="1">
+    <row r="26" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="11">
         <v>20</v>
       </c>
@@ -1393,7 +1540,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
     </row>
-    <row r="27" spans="2:7" ht="31.15" customHeight="1">
+    <row r="27" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="11">
         <v>21</v>
       </c>
@@ -1403,7 +1550,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
-    <row r="28" spans="2:7" ht="31.15" customHeight="1">
+    <row r="28" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="9">
         <v>22</v>
       </c>
@@ -1413,7 +1560,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
-    <row r="30" spans="2:7">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B30" s="19" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Added update_balance and adjusted test_client.py and client.py notes and coding
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_client.xlsx
+++ b/tests/A01_pixell_test_plan_client.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment_01/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{5ECD6C5C-0BF7-4659-811B-1D416A6C1BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D24A0B50-E7AA-48E0-A4DB-DD89C6733701}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{5ECD6C5C-0BF7-4659-811B-1D416A6C1BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04A09CD9-ADD5-4E60-A518-514D622EA767}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19390" windowHeight="15370" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
   <si>
     <t>Software Development Team - Unit Test Plan</t>
   </si>
@@ -269,9 +269,6 @@
     <t>Trevor Donald</t>
   </si>
   <si>
-    <t>ok</t>
-  </si>
-  <si>
     <t>ValueError (""Client Number must be of a numeric type.")</t>
   </si>
   <si>
@@ -284,71 +281,61 @@
     <t>EmailNotValidError ("Email Address not valid")</t>
   </si>
   <si>
-    <t>self.assertEqual( {input},client._Client _client_number / client.Client_first_name / client._Client_last_name / client._client _email_adress)</t>
-  </si>
-  <si>
-    <t>Initializing the class by calling the class with valid inputs example:      Client(123,"Trevor","Donald","tdonald35@academic.rrc.ca")</t>
-  </si>
-  <si>
-    <t>Initializing the class by calling the class with invalid inputs example:      Client("123","Trevor","Donald","tdonald35@academic.rrc.ca")</t>
-  </si>
-  <si>
-    <t>Initializing the class by calling the class with invalid inputs example:      Client(123,"","Donald","tdonald35@academic.rrc.ca")</t>
-  </si>
-  <si>
-    <t>Initializing the class by calling the class with invalid inputs example:      Client(123,"Trevor","","tdonald35@academic.rrc.ca")</t>
-  </si>
-  <si>
-    <t>Initializing the class by calling the class with invalid inputs example:      Client(123,"Trevor","Donald","invalid")</t>
-  </si>
-  <si>
-    <t>After initializing the class calliing the accessor client.client_number</t>
-  </si>
-  <si>
-    <t>After initializing the class calliing the accessor client.first_name</t>
-  </si>
-  <si>
-    <t>After initializing the class calliing the accessor client.last_name</t>
-  </si>
-  <si>
-    <t>After initializing the class calliing the accessor client.email_address</t>
-  </si>
-  <si>
-    <t>After initializing the class calliing the __str__ print(client)</t>
-  </si>
-  <si>
-    <t>self.assertEqual( {input}, self.client.email_adress)</t>
-  </si>
-  <si>
-    <t>self.assertEqual( {input}, self.client.last_name)</t>
-  </si>
-  <si>
-    <t>self.assertEqual( {input}, self.client.first_name)</t>
-  </si>
-  <si>
-    <t>self.assertEqual( {input}, self.client.client_number)</t>
-  </si>
-  <si>
-    <t>self.assertEqual( {input}, str(self.client)</t>
-  </si>
-  <si>
-    <t>with self.assertRaises(ValueError) as context:Client("123", "Trevor", "Donald", "Tdonald35@academic.rrc.ca")
-self.assertEqual(expected, str(context.exception))</t>
-  </si>
-  <si>
-    <t>with self.assertRaises(ValueError) as context:
-            Client(123, "", "Donald", "Tdonald35@academic.rrc.ca")
-        self.assertEqual(expected, str(context.exception))</t>
-  </si>
-  <si>
-    <t>ith self.assertRaises(ValueError) as context:
-            Client(123, "Trevor", "", "Tdonald35@academic.rrc.ca")
-        self.assertEqual(expected, str(context.exception))</t>
-  </si>
-  <si>
-    <t>with self.assertRaises(ValueError) as context:
-            Client(123, "Trevor", "", "Tdonald35@academic.rrc.ca")
-        self.assertEqual(expected, str(context.exception))</t>
+    <t xml:space="preserve">      Client(123,"Trevor","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Client("123","Trevor","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Client(123,"","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Client(123,"Trevor","","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Client(123,"Trevor","Donald","invalid")</t>
+  </si>
+  <si>
+    <t>Client(123,"Trevor","Donald","tdonald35@academic.rrc.ca")</t>
+  </si>
+  <si>
+    <t>client_id = 123</t>
+  </si>
+  <si>
+    <t>client_id = 123                           first_name = "Trevor"                      last_name = "Donald"                 email_address = "tdonald35@academic.rrc.ca"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">client_id = 123                           </t>
+  </si>
+  <si>
+    <t>first_name = "Trevor"</t>
+  </si>
+  <si>
+    <t>last_name = "Donald"</t>
+  </si>
+  <si>
+    <t>email_address = "tdonald35@academic.rrc.ca"</t>
+  </si>
+  <si>
+    <t>"Donald, Trevor, [123] - Tdonald35@academic.rrc.ca"</t>
+  </si>
+  <si>
+    <t>__str___ = "Donald, Trevor, [123] - Tdonald35@academic.rrc.ca"</t>
+  </si>
+  <si>
+    <t>client_id = "123"</t>
+  </si>
+  <si>
+    <t>first_name = ""</t>
+  </si>
+  <si>
+    <t>last_name = ""</t>
+  </si>
+  <si>
+    <t>email_address = "invalid"</t>
+  </si>
+  <si>
+    <t>client_id = 123                                          first_name = "Trevor"                               last_name = "Donald"                 email_address = "tdonald35@academic.rrc.ca"</t>
   </si>
 </sst>
 </file>
@@ -773,6 +760,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1247,13 +1238,13 @@
         <v>11</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
@@ -1268,13 +1259,13 @@
         <v>12</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
@@ -1289,13 +1280,13 @@
         <v>13</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
@@ -1310,13 +1301,13 @@
         <v>14</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.35">
@@ -1331,13 +1322,13 @@
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1351,13 +1342,13 @@
         <v>17</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1371,13 +1362,13 @@
         <v>19</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1391,13 +1382,13 @@
         <v>21</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1411,13 +1402,13 @@
         <v>23</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1431,13 +1422,13 @@
         <v>25</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>28</v>
+        <v>45</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>